<commit_message>
Fix GC filter automation and Memgraph expectations for phs002430
</commit_message>
<xml_diff>
--- a/InputFiles/GC/TC01_GC_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture.xlsx
+++ b/InputFiles/GC/TC01_GC_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture.xlsx
@@ -1,168 +1,54 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sohilz2/Automation/Commons_Automation/InputFiles/CDS/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A79389-6B4C-7648-A6AB-51E24AEBF752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>TabName</t>
-  </si>
-  <si>
-    <t>TabQuery</t>
-  </si>
-  <si>
-    <t>StatQuery</t>
-  </si>
-  <si>
-    <t>TsvExcel</t>
-  </si>
-  <si>
-    <t>WebExcel</t>
-  </si>
-  <si>
-    <t>ParticipantsTab</t>
-  </si>
-  <si>
-    <t>TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture_TSVData.xlsx</t>
-  </si>
-  <si>
-    <t>TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture_WebData.xlsx</t>
-  </si>
-  <si>
-    <t>SamplesTab</t>
-  </si>
-  <si>
-    <t>FilesTab</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
-MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
-WHERE s.phs_accession = "phs002599"
-  AND samp.sample_tumor_status = "Not specified in data"
-  AND samp.sample_type = "RNA"
-RETURN DISTINCT
-  s.study_acronym AS study_name,
-  s.phs_accession AS accession,
-  samp.sample_id AS sample_id,
-  COALESCE(samp.sample_name, samp.sample_id) AS sample_name,
-  COALESCE(samp.Organization_Name, "Not specified in data") AS organization_name
-ORDER BY samp.sample_id ASC
-LIMIT 100
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
-MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
-WHERE s.phs_accession = "phs002599"
-  AND samp.sample_tumor_status = "Not specified in data"
-  AND samp.sample_type = "RNA"
-WITH DISTINCT p, s
-OPTIONAL MATCH (samp_all:sample)-[:of_participant]-&gt;(p)
-WITH p, s, samp_all
-ORDER BY samp_all.sample_id ASC
-WITH p, s, [x IN collect(samp_all.sample_id) WHERE x IS NOT NULL] AS sample_ids
-WITH p, s, sample_ids,
-  CASE
-    WHEN size(sample_ids) &gt; 5
-    THEN reduce(acc = "", id IN sample_ids[0..5] | CASE WHEN acc = "" THEN id ELSE acc + ", " + id END) + ", ..."
-    ELSE reduce(acc = "", id IN sample_ids | CASE WHEN acc = "" THEN id ELSE acc + ", " + id END)
-  END AS samples
-RETURN
-  p.participant_id AS participant_id,
-  s.study_name AS study_name,
-  s.phs_accession AS accession,
-  p.sex AS sex,
-  samples
-ORDER BY p.participant_id ASC
-LIMIT 100
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
-MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
-WHERE s.phs_accession = "phs002599"
-  AND samp.sample_tumor_status = "Not specified in data"
-  AND samp.sample_type = "RNA"
-  RETURN
-  count(DISTINCT s) AS Studies,
-  count(DISTINCT p) AS Participants,
-  count(DISTINCT samp) AS Samples,
-  count(DISTINCT f) AS Files
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
-MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
-MATCH (f)-[:from_sample]-&gt;(samp)
-WHERE s.phs_accession = "phs002599"
-  AND samp.sample_tumor_status = "Not specified in data"
-  AND samp.sample_type = "RNA"
-RETURN DISTINCT
-  s.study_name AS study_name,
-  s.phs_accession AS accession,
-  f.file_name AS file_name,
-  f.file_id AS file_id,
-  f.file_type AS file_type,
-  COALESCE(samp.sample_id, "Not Applicable") AS sample_id
-ORDER BY f.file_name ASC
-LIMIT 100
-</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color indexed="8"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -182,31 +68,90 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -506,74 +451,169 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="75.83203125" customWidth="1"/>
-    <col min="4" max="4" width="87.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="88.6640625" bestFit="1" customWidth="1"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="75.83203125" customWidth="1" min="2" max="3"/>
+    <col width="87.83203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="88.6640625" bestFit="1" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TabName</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TabQuery</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>StatQuery</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>TsvExcel</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>WebExcel</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
+    <row r="2" ht="409.5" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ParticipantsTab</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
+WHERE s.phs_accession = "phs002599"
+  AND samp.sample_tumor_status = "Not specified in data"
+  AND samp.sample_type = "RNA"
+WITH DISTINCT p, s
+OPTIONAL MATCH (samp_all:sample)-[:of_participant]-&gt;(p)
+WITH p, s, samp_all
+ORDER BY samp_all.sample_id ASC
+WITH p, s, [x IN collect(samp_all.sample_id) WHERE x IS NOT NULL] AS sample_ids
+WITH p, s, sample_ids,
+  CASE
+    WHEN size(sample_ids) &gt; 5
+    THEN reduce(acc = "", id IN sample_ids[0..5] | CASE WHEN acc = "" THEN id ELSE acc + ", " + id END) + ", ..."
+    ELSE reduce(acc = "", id IN sample_ids | CASE WHEN acc = "" THEN id ELSE acc + ", " + id END)
+  END AS samples
+RETURN
+  p.participant_id AS participant_id,
+  s.study_name AS study_name,
+  s.phs_accession AS accession,
+  p.sex AS sex,
+  samples
+ORDER BY p.participant_id ASC
+LIMIT 100
+</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
+MATCH (f)-[:from_sample]-&gt;(samp)
+WHERE s.phs_accession = "phs002599"
+  AND samp.sample_tumor_status = "Not specified in data"
+  AND samp.sample_type = "RNA"
+  RETURN
+  count(DISTINCT s) AS Studies,
+  count(DISTINCT p) AS Participants,
+  count(DISTINCT samp) AS Samples,
+  count(DISTINCT f) AS Files
+</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture_TSVData.xlsx</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture_WebData.xlsx</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2"/>
+    <row r="3" ht="409.5" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SamplesTab</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
+WHERE s.phs_accession = "phs002599"
+  AND samp.sample_tumor_status = "Not specified in data"
+  AND samp.sample_type = "RNA"
+RETURN DISTINCT
+  s.study_acronym AS study_name,
+  s.phs_accession AS accession,
+  samp.sample_id AS sample_id,
+  COALESCE(samp.sample_name, samp.sample_id) AS sample_name,
+  COALESCE(samp.Organization_Name, "Not specified in data") AS organization_name
+ORDER BY samp.sample_id ASC
+LIMIT 100
+</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
     </row>
-    <row r="4" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2"/>
+    <row r="4" ht="409.5" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FilesTab</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
+MATCH (f)-[:from_sample]-&gt;(samp)
+WHERE s.phs_accession = "phs002599"
+  AND samp.sample_tumor_status = "Not specified in data"
+  AND samp.sample_type = "RNA"
+RETURN DISTINCT
+  s.study_name AS study_name,
+  s.phs_accession AS accession,
+  f.file_name AS file_name,
+  f.file_id AS file_id,
+  f.file_type AS file_type,
+  COALESCE(samp.sample_id, "Not Applicable") AS sample_id
+ORDER BY f.file_name ASC
+LIMIT 100
+</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
+    <row r="5">
+      <c r="B5" s="1" t="n"/>
+      <c r="C5" s="1" t="n"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C6" s="1"/>
+    <row r="6">
+      <c r="C6" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>